<commit_message>
cotisation avec bareme correspondant, mais NDD cot° not ok
</commit_message>
<xml_diff>
--- a/Template_insertion_adherents.xlsx
+++ b/Template_insertion_adherents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Apps\sebtp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABCB9CA-FF5F-43A3-8F11-FFB58E246691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35910C1-26D9-478E-A38E-050DE5439601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{7D5D9DA3-7695-4AB8-AE95-6DED58FAFFA8}"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{7D5D9DA3-7695-4AB8-AE95-6DED58FAFFA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="66">
   <si>
     <t>email</t>
   </si>
@@ -87,9 +87,6 @@
     <t>actif</t>
   </si>
   <si>
-    <t>OTI</t>
-  </si>
-  <si>
     <t>NIF</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
     <t>statut (radie/actif/inactif/demande)</t>
   </si>
   <si>
-    <t>comm.si@oti.mg</t>
-  </si>
-  <si>
     <t>BTP</t>
   </si>
   <si>
@@ -181,6 +175,54 @@
   </si>
   <si>
     <t>ref@test.com</t>
+  </si>
+  <si>
+    <t>Lot IVJ 163 Ambohimanarina</t>
+  </si>
+  <si>
+    <t>RAMIJOROA Lalaina Kiady Aaron</t>
+  </si>
+  <si>
+    <t>Président du SEBTP</t>
+  </si>
+  <si>
+    <t>aaronkiady77@gmail.com</t>
+  </si>
+  <si>
+    <t>ramijoroaaaron@gmail.com</t>
+  </si>
+  <si>
+    <t>AARON GROUP</t>
+  </si>
+  <si>
+    <t>BTP / Construction</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
+    <t>simple</t>
+  </si>
+  <si>
+    <t>Tresorier du SEBTP</t>
+  </si>
+  <si>
+    <t>Bandy milay</t>
+  </si>
+  <si>
+    <t>entreprise</t>
+  </si>
+  <si>
+    <t>S65S3SFR53</t>
+  </si>
+  <si>
+    <t>REFCNAPS</t>
+  </si>
+  <si>
+    <t>ref@erent.com</t>
+  </si>
+  <si>
+    <t>KIADY</t>
   </si>
 </sst>
 </file>
@@ -583,7 +625,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.44140625" customWidth="1"/>
     <col min="4" max="4" width="26.44140625" customWidth="1"/>
     <col min="5" max="5" width="16.5546875" customWidth="1"/>
@@ -605,6 +647,7 @@
     <col min="21" max="21" width="17.6640625" customWidth="1"/>
     <col min="22" max="22" width="37" customWidth="1"/>
     <col min="23" max="23" width="13.88671875" customWidth="1"/>
+    <col min="24" max="24" width="11" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="11" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="10" bestFit="1" customWidth="1"/>
@@ -631,7 +674,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -649,7 +692,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>10</v>
@@ -658,7 +701,7 @@
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>12</v>
@@ -667,7 +710,7 @@
         <v>13</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>14</v>
@@ -676,77 +719,91 @@
         <v>15</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="X1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Z1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="Z1" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="AA1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AB1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="AD1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AG1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AH1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AG1" s="4" t="s">
+      <c r="AI1" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="AI1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
+        <v>53</v>
+      </c>
+      <c r="B2" s="3">
+        <v>381053233</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="D2" s="3" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H2" s="3"/>
+        <v>44</v>
+      </c>
+      <c r="H2" s="3">
+        <v>20</v>
+      </c>
       <c r="I2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L2" s="3">
+        <v>381053233</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" s="3"/>
+      <c r="N2" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3" t="s">
         <v>19</v>
@@ -758,85 +815,147 @@
         <v>46205</v>
       </c>
       <c r="U2" s="5">
-        <v>41255</v>
+        <v>46215</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3">
         <v>1222222</v>
       </c>
       <c r="Y2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z2" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="AA2" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="AB2" s="3">
-        <v>3800123456</v>
+        <v>380012345</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AE2" s="3">
         <v>380030696</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AG2" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AH2" s="3">
         <v>380030994</v>
       </c>
       <c r="AI2" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
+      <c r="A3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="3">
+        <v>380933982</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="3">
+        <v>5</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="3">
+        <v>381053233</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
+      <c r="P3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
+      <c r="T3" s="5">
+        <v>46223</v>
+      </c>
+      <c r="U3" s="5">
+        <v>46225</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
-      <c r="AE3" s="3"/>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3"/>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3"/>
+      <c r="X3" s="3">
+        <v>2103206510</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>380030440</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>380030696</v>
+      </c>
+      <c r="AF3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AG3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH3" s="3">
+        <v>380030994</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
@@ -918,8 +1037,12 @@
     <hyperlink ref="AF2" r:id="rId2" xr:uid="{F5816441-8416-406A-A6DD-76D1A70EA7E0}"/>
     <hyperlink ref="AI2" r:id="rId3" xr:uid="{A9F4704E-B105-4988-881B-D88BE8E6FA96}"/>
     <hyperlink ref="AC2" r:id="rId4" xr:uid="{D0BB8037-FC9A-491B-962F-B87E02C66E51}"/>
+    <hyperlink ref="A3" r:id="rId5" xr:uid="{2D425FA1-F4A7-4758-AC2A-47ED6BE299F5}"/>
+    <hyperlink ref="AC3" r:id="rId6" xr:uid="{55D8BAFB-AC6D-4F9B-AF4E-02290733D685}"/>
+    <hyperlink ref="AF3" r:id="rId7" xr:uid="{17A7429A-9A0D-419E-A18E-27FFC752101C}"/>
+    <hyperlink ref="AI3" r:id="rId8" xr:uid="{3765F1F7-1A74-43DF-B4DE-A3F7EE07DD92}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>